<commit_message>
chore(preview): TSLA outputs regeneres
</commit_message>
<xml_diff>
--- a/preview/TSLA/TSLA_financials.xlsx
+++ b/preview/TSLA/TSLA_financials.xlsx
@@ -14924,7 +14924,7 @@
         <v>226</v>
       </c>
       <c r="H95" s="238" t="n">
-        <v>376.71</v>
+        <v>375.03</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
@@ -15056,7 +15056,7 @@
       <c r="F100" s="458" t="n"/>
       <c r="G100" s="458" t="n"/>
       <c r="H100" s="459" t="n">
-        <v>0.0433</v>
+        <v>0.0432</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
@@ -15192,7 +15192,7 @@
       <c r="F106" s="458" t="n"/>
       <c r="G106" s="458" t="n"/>
       <c r="H106" s="459" t="n">
-        <v>0.9943</v>
+        <v>0.9942</v>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1">
@@ -15212,7 +15212,7 @@
       <c r="F107" s="458" t="n"/>
       <c r="G107" s="458" t="n"/>
       <c r="H107" s="459" t="n">
-        <v>0.0057</v>
+        <v>0.0058</v>
       </c>
     </row>
     <row r="108" ht="15" customHeight="1">
@@ -15913,7 +15913,7 @@
         </is>
       </c>
       <c r="C15" s="573" t="n">
-        <v>376.71</v>
+        <v>374.99</v>
       </c>
     </row>
     <row r="17">
@@ -26029,7 +26029,7 @@
         </is>
       </c>
       <c r="D9" s="542" t="n">
-        <v>75.3</v>
+        <v>75.03</v>
       </c>
       <c r="E9" s="476" t="n">
         <v>173303.61</v>
@@ -26069,7 +26069,7 @@
         </is>
       </c>
       <c r="D10" s="542" t="n">
-        <v>11.61</v>
+        <v>11.63</v>
       </c>
       <c r="E10" s="476" t="n">
         <v>183371.55</v>
@@ -26189,7 +26189,7 @@
         </is>
       </c>
       <c r="D13" s="543" t="n">
-        <v>87.84</v>
+        <v>87.95999999999999</v>
       </c>
       <c r="E13" s="479" t="n">
         <v>258704.92</v>

</xml_diff>